<commit_message>
B&N rev12 WIP: back-check fixes (no folder names, full head track breakdown), rules R80e.33-35 classified
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev12.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev12.xlsx
@@ -1357,7 +1357,7 @@
     <t xml:space="preserve">Additional head track at openings over 4'-0" wide - extended to every door as a 2-piece track header (R.O. + 1'-4") x 2 (RFI-09)</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: 1/A-500 | Door 14 (W2-01): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 11 (W2-03): (4.0 + 2 x 0.667) x 1 x 2 pieces = 10.67; Door 4 (W2-04): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 9 (W2-06.1): (3.33 + 2 x 0.667) x 1 x 2 pieces = 9.33; Door 8 (W2-06.5): (3.33 + 2 x 0.667) x 1 x 2 pieces = 9.33; Door 7 (W2-06.5): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 5 (W2-08): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 6 (W2-09): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 3 (C-H2a): (4.0 + 2 x 0.667)</t>
+    <t xml:space="preserve">N/SHEET: 1/A-500 | Door 14 (W2-01): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 11 (W2-03): (4.0 + 2 x 0.667) x 1 x 2 pieces = 10.67; Door 4 (W2-04): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 9 (W2-06.1): (3.33 + 2 x 0.667) x 1 x 2 pieces = 9.33; Door 8 (W2-06.5): (3.33 + 2 x 0.667) x 1 x 2 pieces = 9.33; Door 7 (W2-06.5): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 5 (W2-08): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 6 (W2-09): (3.0 + 2 x 0.667) x 1 x 2 pieces = 8.67; Door 3 (C-H2a): (4.0 + 2 x 0.667) x 1 x 2 pieces = 10.67</t>
   </si>
   <si>
     <t xml:space="preserve">Stud reinforcement at MEP penetrations</t>
@@ -1492,7 +1492,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-27: Counted on M-102 + A-101: 8 duct crossings at the full-height walls (types 2 / 5) + 2 TG-1 transfer grille openings (W2-03, W2-02). N/SHEET: M-102; A-101.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: stud reinforcement plates 0 -&gt; 10 (8 ducts x 1 + 2 TG-1); duct sleeves 0 -&gt; 8 (rfi_mep_cruces/CRUCES.md).</t>
+    <t xml:space="preserve">Applied: stud reinforcement plates 0 -&gt; 10 (8 ducts x 1 + 2 TG-1); duct sleeves 0 -&gt; 8.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-01</t>
@@ -1738,7 +1738,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-27: Both: (a) stainless steel corner guard 48" at the corner the C22 leader points to (existing perimeter, the plan asks for it); (b) metal corner guards 2"x2"x72" at all outside corners. N/SHEET: C22/A-101; A-001A.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: stainless 48" = 1; metal 2"x2"x72" = 72 (C25 36, type 3 16, type 4 8, type 2 5, Cafe 7) - rfi29_corner_guards/CONTEO.md.</t>
+    <t xml:space="preserve">Applied: stainless 48" = 1; metal 2"x2"x72" = 72 (C25 36, type 3 16, type 4 8, type 2 5, Cafe 7).</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-30</t>
@@ -1864,7 +1864,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-27: E1 cement board to 12'-0" (TL-4 / WD-1 to 11'-6" on 4/A-226A + 6"; 11'-6" at C-E1-B). N/SHEET: E/A-221; 4/A-226A; 1/A-121.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: 1/2" cement board - 305.62 SF (C-E1-S 19.0 x 13.0 + C-E1-P.2 2.11 x 13.0 + C-E1-B 2.31 x 13.5) - rfi43_cement_board/.</t>
+    <t xml:space="preserve">Applied: 1/2" cement board - 305.62 SF (C-E1-S 19.0 x 13.0 + C-E1-P.2 2.11 x 13.0 + C-E1-B 2.31 x 13.5).</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-44</t>
@@ -1915,7 +1915,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-27: Resolved on the plan: 0 cased openings (A-500 schedule / types; no 2/A-500 bubble on any sheet). "2/A-500 detail not referenced on any plan". N/SHEET: 2/A-500; A-500.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: 2x wood blocking - 17.0 LF (rfi49_cased_openings/).</t>
+    <t xml:space="preserve">Applied: 2x wood blocking - 17.0 LF.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-50</t>
@@ -2272,7 +2272,7 @@
     <t xml:space="preserve">reglas.py compuerta OK</t>
   </si>
   <si>
-    <t xml:space="preserve">{"canon": "54a2985ce868bef5f4c86f781a371493b3c8a301911697047c99b99bfdd32ea4", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "7b57a39cc3c109040dd7d70891acabfb54c970e8bd928b5acae84020f0009372", "reglas": "ba8bd6e1d9f05fc9d972b956fc70d6670e442c3778886e8c3bd2d878c81dab17", "version": "v73"}</t>
+    <t xml:space="preserve">{"canon": "54a2985ce868bef5f4c86f781a371493b3c8a301911697047c99b99bfdd32ea4", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "7b57a39cc3c109040dd7d70891acabfb54c970e8bd928b5acae84020f0009372", "reglas": "26cd43ad2b0dabf9c000cc5efad076b676363c3a45b7af4570136de43fd09305", "version": "v73"}</t>
   </si>
 </sst>
 </file>

</xml_diff>